<commit_message>
G1: refresh importer reports from dynamic-block re-imports
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-adventure-listing.report.xlsx
+++ b/tools/importer/reports/import-adventure-listing.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="314">
   <si>
     <t>_reportFile</t>
   </si>
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-09-22T13:50:57.461Z</t>
+    <t>2026-09-22T13:55:32.070Z</t>
   </si>
   <si>
     <t>WKND Adventures and Travel</t>
@@ -61,6 +61,117 @@
     <t>https://wknd.site/ca/en.html</t>
   </si>
   <si>
+    <t>ca/fr.report.json</t>
+  </si>
+  <si>
+    <t>[]</t>
+  </si>
+  <si>
+    <t>ca/fr</t>
+  </si>
+  <si>
+    <t>2026-09-22T13:55:36.403Z</t>
+  </si>
+  <si>
+    <t>Français</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/fr.html</t>
+  </si>
+  <si>
+    <t>ch/de.report.json</t>
+  </si>
+  <si>
+    <t>ch/de</t>
+  </si>
+  <si>
+    <t>2026-09-22T13:55:41.573Z</t>
+  </si>
+  <si>
+    <t>Deutsch</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ch/de.html</t>
+  </si>
+  <si>
+    <t>ch/fr.report.json</t>
+  </si>
+  <si>
+    <t>ch/fr</t>
+  </si>
+  <si>
+    <t>2026-09-22T13:55:46.517Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ch/fr.html</t>
+  </si>
+  <si>
+    <t>ch/it.report.json</t>
+  </si>
+  <si>
+    <t>ch/it</t>
+  </si>
+  <si>
+    <t>2026-09-22T13:55:53.112Z</t>
+  </si>
+  <si>
+    <t>Italiano</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ch/it.html</t>
+  </si>
+  <si>
+    <t>de/de.report.json</t>
+  </si>
+  <si>
+    <t>de/de</t>
+  </si>
+  <si>
+    <t>2026-09-22T13:55:59.676Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/de/de.html</t>
+  </si>
+  <si>
+    <t>es/es.report.json</t>
+  </si>
+  <si>
+    <t>es/es</t>
+  </si>
+  <si>
+    <t>2026-09-22T13:56:05.297Z</t>
+  </si>
+  <si>
+    <t>Español</t>
+  </si>
+  <si>
+    <t>https://wknd.site/es/es.html</t>
+  </si>
+  <si>
+    <t>fr/fr.report.json</t>
+  </si>
+  <si>
+    <t>fr/fr</t>
+  </si>
+  <si>
+    <t>2026-09-22T13:56:10.881Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/fr/fr.html</t>
+  </si>
+  <si>
+    <t>it/it.report.json</t>
+  </si>
+  <si>
+    <t>it/it</t>
+  </si>
+  <si>
+    <t>2026-09-22T13:56:15.544Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/it/it.html</t>
+  </si>
+  <si>
     <t>us/en.report.json</t>
   </si>
   <si>
@@ -73,6 +184,18 @@
     <t>https://wknd.site/us/en.html</t>
   </si>
   <si>
+    <t>us/es.report.json</t>
+  </si>
+  <si>
+    <t>us/es</t>
+  </si>
+  <si>
+    <t>2026-09-22T13:56:21.188Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/es.html</t>
+  </si>
+  <si>
     <t>ca/en/about-us.report.json</t>
   </si>
   <si>
@@ -97,7 +220,7 @@
     <t>ca/en/adventures.report.json</t>
   </si>
   <si>
-    <t>["hero-banner","tabs-minimal-dark-withimg"]</t>
+    <t>["hero-banner","adventure-tabs"]</t>
   </si>
   <si>
     <t>ca/en/adventures</t>
@@ -106,7 +229,7 @@
     <t>adventure-listing</t>
   </si>
   <si>
-    <t>2026-09-22T13:07:40.660Z</t>
+    <t>2026-09-23T14:43:56.307Z</t>
   </si>
   <si>
     <t>Adventures</t>
@@ -139,13 +262,10 @@
     <t>ca/en/magazine.report.json</t>
   </si>
   <si>
-    <t>[]</t>
-  </si>
-  <si>
     <t>ca/en/magazine</t>
   </si>
   <si>
-    <t>2026-09-22T13:51:02.655Z</t>
+    <t>2026-09-22T13:57:35.177Z</t>
   </si>
   <si>
     <t>Magazine</t>
@@ -154,18 +274,60 @@
     <t>https://wknd.site/ca/en/magazine.html</t>
   </si>
   <si>
+    <t>us/en/about-us.report.json</t>
+  </si>
+  <si>
+    <t>us/en/about-us</t>
+  </si>
+  <si>
+    <t>2026-09-22T13:57:45.746Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/about-us.html</t>
+  </si>
+  <si>
     <t>us/en/adventures.report.json</t>
   </si>
   <si>
     <t>us/en/adventures</t>
   </si>
   <si>
-    <t>2026-09-22T13:51:31.086Z</t>
+    <t>2026-09-23T14:43:52.690Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures.html</t>
   </si>
   <si>
+    <t>us/en/faqs.report.json</t>
+  </si>
+  <si>
+    <t>us/en/faqs</t>
+  </si>
+  <si>
+    <t>2026-09-22T13:51:35.952Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/faqs.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine.report.json</t>
+  </si>
+  <si>
+    <t>["columns-featured","article-feed","hero-banner","hero-banner"]</t>
+  </si>
+  <si>
+    <t>us/en/magazine</t>
+  </si>
+  <si>
+    <t>magazine-listing</t>
+  </si>
+  <si>
+    <t>2026-09-23T14:30:56.550Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine.html</t>
+  </si>
+  <si>
     <t>ca/en/adventures/bali-surf-camp.report.json</t>
   </si>
   <si>
@@ -178,7 +340,7 @@
     <t>adventure-detail</t>
   </si>
   <si>
-    <t>2026-09-22T13:00:29.762Z</t>
+    <t>2026-09-23T11:12:28.555Z</t>
   </si>
   <si>
     <t>Bali Surf Camp</t>
@@ -193,7 +355,7 @@
     <t>ca/en/adventures/beervana-portland</t>
   </si>
   <si>
-    <t>2026-09-22T13:51:12.710Z</t>
+    <t>2026-09-23T11:12:33.029Z</t>
   </si>
   <si>
     <t>Beervana in Portland</t>
@@ -208,7 +370,7 @@
     <t>ca/en/adventures/climbing-new-zealand</t>
   </si>
   <si>
-    <t>2026-09-22T13:51:18.949Z</t>
+    <t>2026-09-23T11:12:38.175Z</t>
   </si>
   <si>
     <t>Climbing New Zealand</t>
@@ -217,6 +379,201 @@
     <t>https://wknd.site/ca/en/adventures/climbing-new-zealand.html</t>
   </si>
   <si>
+    <t>ca/en/adventures/colorado-rock-climbing.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/colorado-rock-climbing</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:12:44.254Z</t>
+  </si>
+  <si>
+    <t>Colorado Rock Climbing</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/colorado-rock-climbing.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/cycling-southern-utah.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/cycling-southern-utah</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:12:49.289Z</t>
+  </si>
+  <si>
+    <t>Cycling Southern Utah</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/cycling-southern-utah.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/cycling-tuscany.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/cycling-tuscany</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:12:56.106Z</t>
+  </si>
+  <si>
+    <t>Cycling Tuscany</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/cycling-tuscany.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/downhill-skiing-wyoming.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/downhill-skiing-wyoming</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:13:00.374Z</t>
+  </si>
+  <si>
+    <t>Downhill Skiing Wyoming</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/downhill-skiing-wyoming.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/gastronomic-marais-tour.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/gastronomic-marais-tour</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:13:05.816Z</t>
+  </si>
+  <si>
+    <t>Gastronomic Marais Tour</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/gastronomic-marais-tour.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/napa-wine-tasting.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/napa-wine-tasting</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:13:11.243Z</t>
+  </si>
+  <si>
+    <t>Napa Wine Tasting</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/napa-wine-tasting.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/riverside-camping-australia.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/riverside-camping-australia</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:13:15.823Z</t>
+  </si>
+  <si>
+    <t>Riverside Camping</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/riverside-camping-australia.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/ski-touring-mont-blanc.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/ski-touring-mont-blanc</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:13:19.952Z</t>
+  </si>
+  <si>
+    <t>Ski Touring Mont Blanc</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/ski-touring-mont-blanc.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/surf-camp-costa-rica.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/surf-camp-costa-rica</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:13:27.781Z</t>
+  </si>
+  <si>
+    <t>Surf Camp in Costa Rica</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/surf-camp-costa-rica.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/tahoe-skiing.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/tahoe-skiing</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:13:33.091Z</t>
+  </si>
+  <si>
+    <t>Tahoe Skiing</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/tahoe-skiing.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/west-coast-cycling.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/west-coast-cycling</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:13:39.038Z</t>
+  </si>
+  <si>
+    <t>West Coast Cycling</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/west-coast-cycling.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/whistler-mountain-biking.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/whistler-mountain-biking</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:13:45.173Z</t>
+  </si>
+  <si>
+    <t>Whistler Mountain Biking</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/whistler-mountain-biking.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/yosemite-backpacking.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/yosemite-backpacking</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:13:51.047Z</t>
+  </si>
+  <si>
+    <t>Yosemite Backpacking</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/yosemite-backpacking.html</t>
+  </si>
+  <si>
     <t>ca/en/magazine/arctic-surfing.report.json</t>
   </si>
   <si>
@@ -229,7 +586,7 @@
     <t>magazine-article</t>
   </si>
   <si>
-    <t>2026-09-22T13:26:17.739Z</t>
+    <t>2026-09-23T11:08:04.610Z</t>
   </si>
   <si>
     <t>Arctic Surfing</t>
@@ -238,19 +595,364 @@
     <t>https://wknd.site/ca/en/magazine/arctic-surfing.html</t>
   </si>
   <si>
+    <t>ca/en/magazine/guide-la-skateparks.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/magazine/guide-la-skateparks</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:08:08.964Z</t>
+  </si>
+  <si>
+    <t>Ultimate Guide to LA Skateparks</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/magazine/guide-la-skateparks.html</t>
+  </si>
+  <si>
     <t>ca/en/magazine/members-only.report.json</t>
   </si>
   <si>
     <t>ca/en/magazine/members-only</t>
   </si>
   <si>
-    <t>2026-09-22T13:51:06.834Z</t>
+    <t>2026-09-22T13:57:40.058Z</t>
   </si>
   <si>
     <t>Members Only</t>
   </si>
   <si>
     <t>https://wknd.site/ca/en/magazine/members-only.html</t>
+  </si>
+  <si>
+    <t>ca/en/magazine/san-diego-surf.report.json</t>
+  </si>
+  <si>
+    <t>["breadcrumbs"]</t>
+  </si>
+  <si>
+    <t>ca/en/magazine/san-diego-surf</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:08:14.878Z</t>
+  </si>
+  <si>
+    <t>San Diego Surf Spots</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/magazine/san-diego-surf.html</t>
+  </si>
+  <si>
+    <t>ca/en/magazine/ski-touring.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/magazine/ski-touring</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:08:20.633Z</t>
+  </si>
+  <si>
+    <t>Ski Touring</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/magazine/ski-touring.html</t>
+  </si>
+  <si>
+    <t>ca/en/magazine/western-australia.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/magazine/western-australia</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:08:26.103Z</t>
+  </si>
+  <si>
+    <t>Western Australia</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/magazine/western-australia.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/bali-surf-camp.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/bali-surf-camp</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:11:06.753Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/bali-surf-camp.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/beervana-portland.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/beervana-portland</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:11:13.301Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/beervana-portland.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/climbing-new-zealand.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/climbing-new-zealand</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:11:18.165Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/climbing-new-zealand.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/colorado-rock-climbing.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/colorado-rock-climbing</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:11:23.619Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/colorado-rock-climbing.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-southern-utah.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-southern-utah</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:11:29.496Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/cycling-southern-utah.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-tuscany.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-tuscany</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:11:34.773Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/cycling-tuscany.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/downhill-skiing-wyoming.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/downhill-skiing-wyoming</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:11:40.072Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/downhill-skiing-wyoming.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/gastronomic-marais-tour.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/gastronomic-marais-tour</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:11:44.368Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/gastronomic-marais-tour.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/napa-wine-tasting.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/napa-wine-tasting</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:11:50.122Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/napa-wine-tasting.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/riverside-camping-australia.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/riverside-camping-australia</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:11:55.587Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/riverside-camping-australia.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/ski-touring-mont-blanc.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/ski-touring-mont-blanc</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:12:00.736Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/ski-touring-mont-blanc.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/surf-camp-costa-rica.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/surf-camp-costa-rica</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:12:05.562Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/surf-camp-costa-rica.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/tahoe-skiing.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/tahoe-skiing</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:12:10.002Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/tahoe-skiing.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/west-coast-cycling.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/west-coast-cycling</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:12:15.208Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/west-coast-cycling.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/whistler-mountain-biking.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/whistler-mountain-biking</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:12:19.705Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/whistler-mountain-biking.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/yosemite-backpacking.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/yosemite-backpacking</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:12:24.490Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/yosemite-backpacking.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine/arctic-surfing.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/arctic-surfing</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:07:38.186Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/arctic-surfing.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine/guide-la-skateparks.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/guide-la-skateparks</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:07:44.217Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/guide-la-skateparks.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine/san-diego-surf.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/san-diego-surf</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:07:50.272Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/san-diego-surf.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine/ski-touring.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/ski-touring</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:07:55.278Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/ski-touring.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine/western-australia.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/western-australia</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:07:59.565Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/western-australia.html</t>
+  </si>
+  <si>
+    <t>ca/en/magazine/members-only/alaskan-adventure.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/magazine/members-only/alaskan-adventure</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:08:32.439Z</t>
+  </si>
+  <si>
+    <t>Alaskan Adventure</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/magazine/members-only/alaskan-adventure.html</t>
+  </si>
+  <si>
+    <t>ca/en/magazine/members-only/fly-fishing-the-amazon.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/magazine/members-only/fly-fishing-the-amazon</t>
+  </si>
+  <si>
+    <t>2026-09-23T11:08:37.565Z</t>
+  </si>
+  <si>
+    <t>Fly Fishing the Amazon</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/magazine/members-only/fly-fishing-the-amazon.html</t>
   </si>
 </sst>
 </file>
@@ -639,14 +1341,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="39" customWidth="1"/>
+    <col min="1" max="3" width="50" customWidth="1"/>
     <col min="5" max="5" width="19" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="28" customWidth="1"/>
+    <col min="7" max="7" width="33" customWidth="1"/>
     <col min="8" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
@@ -707,10 +1408,10 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D3" t="s">
         <v>11</v>
@@ -719,30 +1420,30 @@
         <v>12</v>
       </c>
       <c r="F3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G3" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="H3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D4" t="s">
         <v>11</v>
       </c>
       <c r="E4" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="F4" t="s">
         <v>24</v>
@@ -759,233 +1460,1585 @@
         <v>27</v>
       </c>
       <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" t="s">
         <v>28</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" t="s">
         <v>29</v>
       </c>
-      <c r="D5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" t="s">
+      <c r="G5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H5" t="s">
         <v>30</v>
-      </c>
-      <c r="F5" t="s">
-        <v>31</v>
-      </c>
-      <c r="G5" t="s">
-        <v>32</v>
-      </c>
-      <c r="H5" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" t="s">
         <v>34</v>
       </c>
-      <c r="B6" t="s">
+      <c r="H6" t="s">
         <v>35</v>
-      </c>
-      <c r="C6" t="s">
-        <v>36</v>
-      </c>
-      <c r="D6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" t="s">
-        <v>37</v>
-      </c>
-      <c r="F6" t="s">
-        <v>38</v>
-      </c>
-      <c r="G6" t="s">
-        <v>39</v>
-      </c>
-      <c r="H6" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B7" t="s">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="D7" t="s">
         <v>11</v>
       </c>
       <c r="E7" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="F7" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="G7" t="s">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="H7" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="C8" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="D8" t="s">
         <v>11</v>
       </c>
       <c r="E8" t="s">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="F8" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="G8" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="H8" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="B9" t="s">
-        <v>52</v>
+        <v>17</v>
       </c>
       <c r="C9" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
       </c>
       <c r="E9" t="s">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="F9" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="G9" t="s">
-        <v>56</v>
+        <v>20</v>
       </c>
       <c r="H9" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="B10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" t="s">
+        <v>51</v>
+      </c>
+      <c r="G10" t="s">
+        <v>34</v>
+      </c>
+      <c r="H10" t="s">
         <v>52</v>
-      </c>
-      <c r="C10" t="s">
-        <v>59</v>
-      </c>
-      <c r="D10" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" t="s">
-        <v>54</v>
-      </c>
-      <c r="F10" t="s">
-        <v>60</v>
-      </c>
-      <c r="G10" t="s">
-        <v>61</v>
-      </c>
-      <c r="H10" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="B11" t="s">
-        <v>52</v>
+        <v>9</v>
       </c>
       <c r="C11" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="D11" t="s">
         <v>11</v>
       </c>
       <c r="E11" t="s">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="F11" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="G11" t="s">
-        <v>66</v>
+        <v>14</v>
       </c>
       <c r="H11" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="B12" t="s">
-        <v>69</v>
+        <v>17</v>
       </c>
       <c r="C12" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="D12" t="s">
         <v>11</v>
       </c>
       <c r="E12" t="s">
-        <v>71</v>
+        <v>12</v>
       </c>
       <c r="F12" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="G12" t="s">
-        <v>73</v>
+        <v>43</v>
       </c>
       <c r="H12" t="s">
-        <v>74</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>61</v>
+      </c>
+      <c r="B13" t="s">
+        <v>62</v>
+      </c>
+      <c r="C13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>64</v>
+      </c>
+      <c r="F13" t="s">
+        <v>65</v>
+      </c>
+      <c r="G13" t="s">
+        <v>66</v>
+      </c>
+      <c r="H13" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>68</v>
+      </c>
+      <c r="B14" t="s">
+        <v>69</v>
+      </c>
+      <c r="C14" t="s">
+        <v>70</v>
+      </c>
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
+        <v>71</v>
+      </c>
+      <c r="F14" t="s">
+        <v>72</v>
+      </c>
+      <c r="G14" t="s">
+        <v>73</v>
+      </c>
+      <c r="H14" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>75</v>
       </c>
-      <c r="B13" t="s">
-        <v>42</v>
-      </c>
-      <c r="C13" t="s">
+      <c r="B15" t="s">
         <v>76</v>
       </c>
-      <c r="D13" t="s">
-        <v>11</v>
-      </c>
-      <c r="E13" t="s">
-        <v>23</v>
-      </c>
-      <c r="F13" t="s">
+      <c r="C15" t="s">
         <v>77</v>
       </c>
-      <c r="G13" t="s">
+      <c r="D15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" t="s">
         <v>78</v>
       </c>
-      <c r="H13" t="s">
+      <c r="F15" t="s">
         <v>79</v>
+      </c>
+      <c r="G15" t="s">
+        <v>80</v>
+      </c>
+      <c r="H15" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>82</v>
+      </c>
+      <c r="B16" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" t="s">
+        <v>83</v>
+      </c>
+      <c r="D16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" t="s">
+        <v>64</v>
+      </c>
+      <c r="F16" t="s">
+        <v>84</v>
+      </c>
+      <c r="G16" t="s">
+        <v>85</v>
+      </c>
+      <c r="H16" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>87</v>
+      </c>
+      <c r="B17" t="s">
+        <v>62</v>
+      </c>
+      <c r="C17" t="s">
+        <v>88</v>
+      </c>
+      <c r="D17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" t="s">
+        <v>64</v>
+      </c>
+      <c r="F17" t="s">
+        <v>89</v>
+      </c>
+      <c r="G17" t="s">
+        <v>66</v>
+      </c>
+      <c r="H17" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>91</v>
+      </c>
+      <c r="B18" t="s">
+        <v>69</v>
+      </c>
+      <c r="C18" t="s">
+        <v>92</v>
+      </c>
+      <c r="D18" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" t="s">
+        <v>71</v>
+      </c>
+      <c r="F18" t="s">
+        <v>93</v>
+      </c>
+      <c r="G18" t="s">
+        <v>73</v>
+      </c>
+      <c r="H18" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>95</v>
+      </c>
+      <c r="B19" t="s">
+        <v>76</v>
+      </c>
+      <c r="C19" t="s">
+        <v>96</v>
+      </c>
+      <c r="D19" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" t="s">
+        <v>78</v>
+      </c>
+      <c r="F19" t="s">
+        <v>97</v>
+      </c>
+      <c r="G19" t="s">
+        <v>80</v>
+      </c>
+      <c r="H19" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>99</v>
+      </c>
+      <c r="B20" t="s">
+        <v>100</v>
+      </c>
+      <c r="C20" t="s">
+        <v>101</v>
+      </c>
+      <c r="D20" t="s">
+        <v>11</v>
+      </c>
+      <c r="E20" t="s">
+        <v>102</v>
+      </c>
+      <c r="F20" t="s">
+        <v>103</v>
+      </c>
+      <c r="G20" t="s">
+        <v>85</v>
+      </c>
+      <c r="H20" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>105</v>
+      </c>
+      <c r="B21" t="s">
+        <v>106</v>
+      </c>
+      <c r="C21" t="s">
+        <v>107</v>
+      </c>
+      <c r="D21" t="s">
+        <v>11</v>
+      </c>
+      <c r="E21" t="s">
+        <v>108</v>
+      </c>
+      <c r="F21" t="s">
+        <v>109</v>
+      </c>
+      <c r="G21" t="s">
+        <v>110</v>
+      </c>
+      <c r="H21" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>112</v>
+      </c>
+      <c r="B22" t="s">
+        <v>106</v>
+      </c>
+      <c r="C22" t="s">
+        <v>113</v>
+      </c>
+      <c r="D22" t="s">
+        <v>11</v>
+      </c>
+      <c r="E22" t="s">
+        <v>108</v>
+      </c>
+      <c r="F22" t="s">
+        <v>114</v>
+      </c>
+      <c r="G22" t="s">
+        <v>115</v>
+      </c>
+      <c r="H22" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>117</v>
+      </c>
+      <c r="B23" t="s">
+        <v>106</v>
+      </c>
+      <c r="C23" t="s">
+        <v>118</v>
+      </c>
+      <c r="D23" t="s">
+        <v>11</v>
+      </c>
+      <c r="E23" t="s">
+        <v>108</v>
+      </c>
+      <c r="F23" t="s">
+        <v>119</v>
+      </c>
+      <c r="G23" t="s">
+        <v>120</v>
+      </c>
+      <c r="H23" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>122</v>
+      </c>
+      <c r="B24" t="s">
+        <v>106</v>
+      </c>
+      <c r="C24" t="s">
+        <v>123</v>
+      </c>
+      <c r="D24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E24" t="s">
+        <v>108</v>
+      </c>
+      <c r="F24" t="s">
+        <v>124</v>
+      </c>
+      <c r="G24" t="s">
+        <v>125</v>
+      </c>
+      <c r="H24" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>127</v>
+      </c>
+      <c r="B25" t="s">
+        <v>106</v>
+      </c>
+      <c r="C25" t="s">
+        <v>128</v>
+      </c>
+      <c r="D25" t="s">
+        <v>11</v>
+      </c>
+      <c r="E25" t="s">
+        <v>108</v>
+      </c>
+      <c r="F25" t="s">
+        <v>129</v>
+      </c>
+      <c r="G25" t="s">
+        <v>130</v>
+      </c>
+      <c r="H25" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>132</v>
+      </c>
+      <c r="B26" t="s">
+        <v>106</v>
+      </c>
+      <c r="C26" t="s">
+        <v>133</v>
+      </c>
+      <c r="D26" t="s">
+        <v>11</v>
+      </c>
+      <c r="E26" t="s">
+        <v>108</v>
+      </c>
+      <c r="F26" t="s">
+        <v>134</v>
+      </c>
+      <c r="G26" t="s">
+        <v>135</v>
+      </c>
+      <c r="H26" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>137</v>
+      </c>
+      <c r="B27" t="s">
+        <v>106</v>
+      </c>
+      <c r="C27" t="s">
+        <v>138</v>
+      </c>
+      <c r="D27" t="s">
+        <v>11</v>
+      </c>
+      <c r="E27" t="s">
+        <v>108</v>
+      </c>
+      <c r="F27" t="s">
+        <v>139</v>
+      </c>
+      <c r="G27" t="s">
+        <v>140</v>
+      </c>
+      <c r="H27" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>142</v>
+      </c>
+      <c r="B28" t="s">
+        <v>106</v>
+      </c>
+      <c r="C28" t="s">
+        <v>143</v>
+      </c>
+      <c r="D28" t="s">
+        <v>11</v>
+      </c>
+      <c r="E28" t="s">
+        <v>108</v>
+      </c>
+      <c r="F28" t="s">
+        <v>144</v>
+      </c>
+      <c r="G28" t="s">
+        <v>145</v>
+      </c>
+      <c r="H28" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>147</v>
+      </c>
+      <c r="B29" t="s">
+        <v>106</v>
+      </c>
+      <c r="C29" t="s">
+        <v>148</v>
+      </c>
+      <c r="D29" t="s">
+        <v>11</v>
+      </c>
+      <c r="E29" t="s">
+        <v>108</v>
+      </c>
+      <c r="F29" t="s">
+        <v>149</v>
+      </c>
+      <c r="G29" t="s">
+        <v>150</v>
+      </c>
+      <c r="H29" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>152</v>
+      </c>
+      <c r="B30" t="s">
+        <v>106</v>
+      </c>
+      <c r="C30" t="s">
+        <v>153</v>
+      </c>
+      <c r="D30" t="s">
+        <v>11</v>
+      </c>
+      <c r="E30" t="s">
+        <v>108</v>
+      </c>
+      <c r="F30" t="s">
+        <v>154</v>
+      </c>
+      <c r="G30" t="s">
+        <v>155</v>
+      </c>
+      <c r="H30" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>157</v>
+      </c>
+      <c r="B31" t="s">
+        <v>106</v>
+      </c>
+      <c r="C31" t="s">
+        <v>158</v>
+      </c>
+      <c r="D31" t="s">
+        <v>11</v>
+      </c>
+      <c r="E31" t="s">
+        <v>108</v>
+      </c>
+      <c r="F31" t="s">
+        <v>159</v>
+      </c>
+      <c r="G31" t="s">
+        <v>160</v>
+      </c>
+      <c r="H31" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>162</v>
+      </c>
+      <c r="B32" t="s">
+        <v>106</v>
+      </c>
+      <c r="C32" t="s">
+        <v>163</v>
+      </c>
+      <c r="D32" t="s">
+        <v>11</v>
+      </c>
+      <c r="E32" t="s">
+        <v>108</v>
+      </c>
+      <c r="F32" t="s">
+        <v>164</v>
+      </c>
+      <c r="G32" t="s">
+        <v>165</v>
+      </c>
+      <c r="H32" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>167</v>
+      </c>
+      <c r="B33" t="s">
+        <v>106</v>
+      </c>
+      <c r="C33" t="s">
+        <v>168</v>
+      </c>
+      <c r="D33" t="s">
+        <v>11</v>
+      </c>
+      <c r="E33" t="s">
+        <v>108</v>
+      </c>
+      <c r="F33" t="s">
+        <v>169</v>
+      </c>
+      <c r="G33" t="s">
+        <v>170</v>
+      </c>
+      <c r="H33" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>172</v>
+      </c>
+      <c r="B34" t="s">
+        <v>106</v>
+      </c>
+      <c r="C34" t="s">
+        <v>173</v>
+      </c>
+      <c r="D34" t="s">
+        <v>11</v>
+      </c>
+      <c r="E34" t="s">
+        <v>108</v>
+      </c>
+      <c r="F34" t="s">
+        <v>174</v>
+      </c>
+      <c r="G34" t="s">
+        <v>175</v>
+      </c>
+      <c r="H34" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>177</v>
+      </c>
+      <c r="B35" t="s">
+        <v>106</v>
+      </c>
+      <c r="C35" t="s">
+        <v>178</v>
+      </c>
+      <c r="D35" t="s">
+        <v>11</v>
+      </c>
+      <c r="E35" t="s">
+        <v>108</v>
+      </c>
+      <c r="F35" t="s">
+        <v>179</v>
+      </c>
+      <c r="G35" t="s">
+        <v>180</v>
+      </c>
+      <c r="H35" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>182</v>
+      </c>
+      <c r="B36" t="s">
+        <v>106</v>
+      </c>
+      <c r="C36" t="s">
+        <v>183</v>
+      </c>
+      <c r="D36" t="s">
+        <v>11</v>
+      </c>
+      <c r="E36" t="s">
+        <v>108</v>
+      </c>
+      <c r="F36" t="s">
+        <v>184</v>
+      </c>
+      <c r="G36" t="s">
+        <v>185</v>
+      </c>
+      <c r="H36" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>187</v>
+      </c>
+      <c r="B37" t="s">
+        <v>188</v>
+      </c>
+      <c r="C37" t="s">
+        <v>189</v>
+      </c>
+      <c r="D37" t="s">
+        <v>11</v>
+      </c>
+      <c r="E37" t="s">
+        <v>190</v>
+      </c>
+      <c r="F37" t="s">
+        <v>191</v>
+      </c>
+      <c r="G37" t="s">
+        <v>192</v>
+      </c>
+      <c r="H37" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>194</v>
+      </c>
+      <c r="B38" t="s">
+        <v>188</v>
+      </c>
+      <c r="C38" t="s">
+        <v>195</v>
+      </c>
+      <c r="D38" t="s">
+        <v>11</v>
+      </c>
+      <c r="E38" t="s">
+        <v>190</v>
+      </c>
+      <c r="F38" t="s">
+        <v>196</v>
+      </c>
+      <c r="G38" t="s">
+        <v>197</v>
+      </c>
+      <c r="H38" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>199</v>
+      </c>
+      <c r="B39" t="s">
+        <v>17</v>
+      </c>
+      <c r="C39" t="s">
+        <v>200</v>
+      </c>
+      <c r="D39" t="s">
+        <v>11</v>
+      </c>
+      <c r="E39" t="s">
+        <v>64</v>
+      </c>
+      <c r="F39" t="s">
+        <v>201</v>
+      </c>
+      <c r="G39" t="s">
+        <v>202</v>
+      </c>
+      <c r="H39" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>204</v>
+      </c>
+      <c r="B40" t="s">
+        <v>205</v>
+      </c>
+      <c r="C40" t="s">
+        <v>206</v>
+      </c>
+      <c r="D40" t="s">
+        <v>11</v>
+      </c>
+      <c r="E40" t="s">
+        <v>190</v>
+      </c>
+      <c r="F40" t="s">
+        <v>207</v>
+      </c>
+      <c r="G40" t="s">
+        <v>208</v>
+      </c>
+      <c r="H40" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>210</v>
+      </c>
+      <c r="B41" t="s">
+        <v>188</v>
+      </c>
+      <c r="C41" t="s">
+        <v>211</v>
+      </c>
+      <c r="D41" t="s">
+        <v>11</v>
+      </c>
+      <c r="E41" t="s">
+        <v>190</v>
+      </c>
+      <c r="F41" t="s">
+        <v>212</v>
+      </c>
+      <c r="G41" t="s">
+        <v>213</v>
+      </c>
+      <c r="H41" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>215</v>
+      </c>
+      <c r="B42" t="s">
+        <v>188</v>
+      </c>
+      <c r="C42" t="s">
+        <v>216</v>
+      </c>
+      <c r="D42" t="s">
+        <v>11</v>
+      </c>
+      <c r="E42" t="s">
+        <v>190</v>
+      </c>
+      <c r="F42" t="s">
+        <v>217</v>
+      </c>
+      <c r="G42" t="s">
+        <v>218</v>
+      </c>
+      <c r="H42" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>220</v>
+      </c>
+      <c r="B43" t="s">
+        <v>106</v>
+      </c>
+      <c r="C43" t="s">
+        <v>221</v>
+      </c>
+      <c r="D43" t="s">
+        <v>11</v>
+      </c>
+      <c r="E43" t="s">
+        <v>108</v>
+      </c>
+      <c r="F43" t="s">
+        <v>222</v>
+      </c>
+      <c r="G43" t="s">
+        <v>110</v>
+      </c>
+      <c r="H43" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>224</v>
+      </c>
+      <c r="B44" t="s">
+        <v>106</v>
+      </c>
+      <c r="C44" t="s">
+        <v>225</v>
+      </c>
+      <c r="D44" t="s">
+        <v>11</v>
+      </c>
+      <c r="E44" t="s">
+        <v>108</v>
+      </c>
+      <c r="F44" t="s">
+        <v>226</v>
+      </c>
+      <c r="G44" t="s">
+        <v>115</v>
+      </c>
+      <c r="H44" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>228</v>
+      </c>
+      <c r="B45" t="s">
+        <v>106</v>
+      </c>
+      <c r="C45" t="s">
+        <v>229</v>
+      </c>
+      <c r="D45" t="s">
+        <v>11</v>
+      </c>
+      <c r="E45" t="s">
+        <v>108</v>
+      </c>
+      <c r="F45" t="s">
+        <v>230</v>
+      </c>
+      <c r="G45" t="s">
+        <v>120</v>
+      </c>
+      <c r="H45" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>232</v>
+      </c>
+      <c r="B46" t="s">
+        <v>106</v>
+      </c>
+      <c r="C46" t="s">
+        <v>233</v>
+      </c>
+      <c r="D46" t="s">
+        <v>11</v>
+      </c>
+      <c r="E46" t="s">
+        <v>108</v>
+      </c>
+      <c r="F46" t="s">
+        <v>234</v>
+      </c>
+      <c r="G46" t="s">
+        <v>125</v>
+      </c>
+      <c r="H46" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>236</v>
+      </c>
+      <c r="B47" t="s">
+        <v>106</v>
+      </c>
+      <c r="C47" t="s">
+        <v>237</v>
+      </c>
+      <c r="D47" t="s">
+        <v>11</v>
+      </c>
+      <c r="E47" t="s">
+        <v>108</v>
+      </c>
+      <c r="F47" t="s">
+        <v>238</v>
+      </c>
+      <c r="G47" t="s">
+        <v>130</v>
+      </c>
+      <c r="H47" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>240</v>
+      </c>
+      <c r="B48" t="s">
+        <v>106</v>
+      </c>
+      <c r="C48" t="s">
+        <v>241</v>
+      </c>
+      <c r="D48" t="s">
+        <v>11</v>
+      </c>
+      <c r="E48" t="s">
+        <v>108</v>
+      </c>
+      <c r="F48" t="s">
+        <v>242</v>
+      </c>
+      <c r="G48" t="s">
+        <v>135</v>
+      </c>
+      <c r="H48" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>244</v>
+      </c>
+      <c r="B49" t="s">
+        <v>106</v>
+      </c>
+      <c r="C49" t="s">
+        <v>245</v>
+      </c>
+      <c r="D49" t="s">
+        <v>11</v>
+      </c>
+      <c r="E49" t="s">
+        <v>108</v>
+      </c>
+      <c r="F49" t="s">
+        <v>246</v>
+      </c>
+      <c r="G49" t="s">
+        <v>140</v>
+      </c>
+      <c r="H49" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>248</v>
+      </c>
+      <c r="B50" t="s">
+        <v>106</v>
+      </c>
+      <c r="C50" t="s">
+        <v>249</v>
+      </c>
+      <c r="D50" t="s">
+        <v>11</v>
+      </c>
+      <c r="E50" t="s">
+        <v>108</v>
+      </c>
+      <c r="F50" t="s">
+        <v>250</v>
+      </c>
+      <c r="G50" t="s">
+        <v>145</v>
+      </c>
+      <c r="H50" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>252</v>
+      </c>
+      <c r="B51" t="s">
+        <v>106</v>
+      </c>
+      <c r="C51" t="s">
+        <v>253</v>
+      </c>
+      <c r="D51" t="s">
+        <v>11</v>
+      </c>
+      <c r="E51" t="s">
+        <v>108</v>
+      </c>
+      <c r="F51" t="s">
+        <v>254</v>
+      </c>
+      <c r="G51" t="s">
+        <v>150</v>
+      </c>
+      <c r="H51" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>256</v>
+      </c>
+      <c r="B52" t="s">
+        <v>106</v>
+      </c>
+      <c r="C52" t="s">
+        <v>257</v>
+      </c>
+      <c r="D52" t="s">
+        <v>11</v>
+      </c>
+      <c r="E52" t="s">
+        <v>108</v>
+      </c>
+      <c r="F52" t="s">
+        <v>258</v>
+      </c>
+      <c r="G52" t="s">
+        <v>155</v>
+      </c>
+      <c r="H52" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>260</v>
+      </c>
+      <c r="B53" t="s">
+        <v>106</v>
+      </c>
+      <c r="C53" t="s">
+        <v>261</v>
+      </c>
+      <c r="D53" t="s">
+        <v>11</v>
+      </c>
+      <c r="E53" t="s">
+        <v>108</v>
+      </c>
+      <c r="F53" t="s">
+        <v>262</v>
+      </c>
+      <c r="G53" t="s">
+        <v>160</v>
+      </c>
+      <c r="H53" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>264</v>
+      </c>
+      <c r="B54" t="s">
+        <v>106</v>
+      </c>
+      <c r="C54" t="s">
+        <v>265</v>
+      </c>
+      <c r="D54" t="s">
+        <v>11</v>
+      </c>
+      <c r="E54" t="s">
+        <v>108</v>
+      </c>
+      <c r="F54" t="s">
+        <v>266</v>
+      </c>
+      <c r="G54" t="s">
+        <v>165</v>
+      </c>
+      <c r="H54" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>268</v>
+      </c>
+      <c r="B55" t="s">
+        <v>106</v>
+      </c>
+      <c r="C55" t="s">
+        <v>269</v>
+      </c>
+      <c r="D55" t="s">
+        <v>11</v>
+      </c>
+      <c r="E55" t="s">
+        <v>108</v>
+      </c>
+      <c r="F55" t="s">
+        <v>270</v>
+      </c>
+      <c r="G55" t="s">
+        <v>170</v>
+      </c>
+      <c r="H55" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>272</v>
+      </c>
+      <c r="B56" t="s">
+        <v>106</v>
+      </c>
+      <c r="C56" t="s">
+        <v>273</v>
+      </c>
+      <c r="D56" t="s">
+        <v>11</v>
+      </c>
+      <c r="E56" t="s">
+        <v>108</v>
+      </c>
+      <c r="F56" t="s">
+        <v>274</v>
+      </c>
+      <c r="G56" t="s">
+        <v>175</v>
+      </c>
+      <c r="H56" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>276</v>
+      </c>
+      <c r="B57" t="s">
+        <v>106</v>
+      </c>
+      <c r="C57" t="s">
+        <v>277</v>
+      </c>
+      <c r="D57" t="s">
+        <v>11</v>
+      </c>
+      <c r="E57" t="s">
+        <v>108</v>
+      </c>
+      <c r="F57" t="s">
+        <v>278</v>
+      </c>
+      <c r="G57" t="s">
+        <v>180</v>
+      </c>
+      <c r="H57" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>280</v>
+      </c>
+      <c r="B58" t="s">
+        <v>106</v>
+      </c>
+      <c r="C58" t="s">
+        <v>281</v>
+      </c>
+      <c r="D58" t="s">
+        <v>11</v>
+      </c>
+      <c r="E58" t="s">
+        <v>108</v>
+      </c>
+      <c r="F58" t="s">
+        <v>282</v>
+      </c>
+      <c r="G58" t="s">
+        <v>185</v>
+      </c>
+      <c r="H58" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>284</v>
+      </c>
+      <c r="B59" t="s">
+        <v>188</v>
+      </c>
+      <c r="C59" t="s">
+        <v>285</v>
+      </c>
+      <c r="D59" t="s">
+        <v>11</v>
+      </c>
+      <c r="E59" t="s">
+        <v>190</v>
+      </c>
+      <c r="F59" t="s">
+        <v>286</v>
+      </c>
+      <c r="G59" t="s">
+        <v>192</v>
+      </c>
+      <c r="H59" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>288</v>
+      </c>
+      <c r="B60" t="s">
+        <v>188</v>
+      </c>
+      <c r="C60" t="s">
+        <v>289</v>
+      </c>
+      <c r="D60" t="s">
+        <v>11</v>
+      </c>
+      <c r="E60" t="s">
+        <v>190</v>
+      </c>
+      <c r="F60" t="s">
+        <v>290</v>
+      </c>
+      <c r="G60" t="s">
+        <v>197</v>
+      </c>
+      <c r="H60" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>292</v>
+      </c>
+      <c r="B61" t="s">
+        <v>205</v>
+      </c>
+      <c r="C61" t="s">
+        <v>293</v>
+      </c>
+      <c r="D61" t="s">
+        <v>11</v>
+      </c>
+      <c r="E61" t="s">
+        <v>190</v>
+      </c>
+      <c r="F61" t="s">
+        <v>294</v>
+      </c>
+      <c r="G61" t="s">
+        <v>208</v>
+      </c>
+      <c r="H61" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>296</v>
+      </c>
+      <c r="B62" t="s">
+        <v>188</v>
+      </c>
+      <c r="C62" t="s">
+        <v>297</v>
+      </c>
+      <c r="D62" t="s">
+        <v>11</v>
+      </c>
+      <c r="E62" t="s">
+        <v>190</v>
+      </c>
+      <c r="F62" t="s">
+        <v>298</v>
+      </c>
+      <c r="G62" t="s">
+        <v>213</v>
+      </c>
+      <c r="H62" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>300</v>
+      </c>
+      <c r="B63" t="s">
+        <v>188</v>
+      </c>
+      <c r="C63" t="s">
+        <v>301</v>
+      </c>
+      <c r="D63" t="s">
+        <v>11</v>
+      </c>
+      <c r="E63" t="s">
+        <v>190</v>
+      </c>
+      <c r="F63" t="s">
+        <v>302</v>
+      </c>
+      <c r="G63" t="s">
+        <v>218</v>
+      </c>
+      <c r="H63" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>304</v>
+      </c>
+      <c r="B64" t="s">
+        <v>188</v>
+      </c>
+      <c r="C64" t="s">
+        <v>305</v>
+      </c>
+      <c r="D64" t="s">
+        <v>11</v>
+      </c>
+      <c r="E64" t="s">
+        <v>190</v>
+      </c>
+      <c r="F64" t="s">
+        <v>306</v>
+      </c>
+      <c r="G64" t="s">
+        <v>307</v>
+      </c>
+      <c r="H64" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>309</v>
+      </c>
+      <c r="B65" t="s">
+        <v>205</v>
+      </c>
+      <c r="C65" t="s">
+        <v>310</v>
+      </c>
+      <c r="D65" t="s">
+        <v>11</v>
+      </c>
+      <c r="E65" t="s">
+        <v>190</v>
+      </c>
+      <c r="F65" t="s">
+        <v>311</v>
+      </c>
+      <c r="G65" t="s">
+        <v>312</v>
+      </c>
+      <c r="H65" t="s">
+        <v>313</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: refresh import reports after content re-import
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-adventure-listing.report.xlsx
+++ b/tools/importer/reports/import-adventure-listing.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="314">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="315">
   <si>
     <t>_reportFile</t>
   </si>
@@ -175,10 +175,13 @@
     <t>us/en.report.json</t>
   </si>
   <si>
+    <t>["carousel-hero","columns-featured","article-feed","article-feed","hero-banner"]</t>
+  </si>
+  <si>
     <t>us/en</t>
   </si>
   <si>
-    <t>2026-09-22T12:35:41.404Z</t>
+    <t>2026-09-24T09:47:30.763Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en.html</t>
@@ -229,7 +232,7 @@
     <t>adventure-listing</t>
   </si>
   <si>
-    <t>2026-09-23T14:43:56.307Z</t>
+    <t>2026-09-24T09:47:47.182Z</t>
   </si>
   <si>
     <t>Adventures</t>
@@ -292,7 +295,7 @@
     <t>us/en/adventures</t>
   </si>
   <si>
-    <t>2026-09-23T14:43:52.690Z</t>
+    <t>2026-09-24T09:47:42.900Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures.html</t>
@@ -322,7 +325,7 @@
     <t>magazine-listing</t>
   </si>
   <si>
-    <t>2026-09-23T14:30:56.550Z</t>
+    <t>2026-09-24T09:47:37.015Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/magazine.html</t>
@@ -340,7 +343,7 @@
     <t>adventure-detail</t>
   </si>
   <si>
-    <t>2026-09-23T11:12:28.555Z</t>
+    <t>2026-09-23T14:52:29.097Z</t>
   </si>
   <si>
     <t>Bali Surf Camp</t>
@@ -355,7 +358,7 @@
     <t>ca/en/adventures/beervana-portland</t>
   </si>
   <si>
-    <t>2026-09-23T11:12:33.029Z</t>
+    <t>2026-09-23T14:52:34.934Z</t>
   </si>
   <si>
     <t>Beervana in Portland</t>
@@ -370,7 +373,7 @@
     <t>ca/en/adventures/climbing-new-zealand</t>
   </si>
   <si>
-    <t>2026-09-23T11:12:38.175Z</t>
+    <t>2026-09-23T14:52:42.206Z</t>
   </si>
   <si>
     <t>Climbing New Zealand</t>
@@ -385,7 +388,7 @@
     <t>ca/en/adventures/colorado-rock-climbing</t>
   </si>
   <si>
-    <t>2026-09-23T11:12:44.254Z</t>
+    <t>2026-09-23T14:52:47.147Z</t>
   </si>
   <si>
     <t>Colorado Rock Climbing</t>
@@ -400,7 +403,7 @@
     <t>ca/en/adventures/cycling-southern-utah</t>
   </si>
   <si>
-    <t>2026-09-23T11:12:49.289Z</t>
+    <t>2026-09-23T14:52:53.189Z</t>
   </si>
   <si>
     <t>Cycling Southern Utah</t>
@@ -415,7 +418,7 @@
     <t>ca/en/adventures/cycling-tuscany</t>
   </si>
   <si>
-    <t>2026-09-23T11:12:56.106Z</t>
+    <t>2026-09-23T14:52:59.133Z</t>
   </si>
   <si>
     <t>Cycling Tuscany</t>
@@ -430,7 +433,7 @@
     <t>ca/en/adventures/downhill-skiing-wyoming</t>
   </si>
   <si>
-    <t>2026-09-23T11:13:00.374Z</t>
+    <t>2026-09-23T14:53:04.577Z</t>
   </si>
   <si>
     <t>Downhill Skiing Wyoming</t>
@@ -445,7 +448,7 @@
     <t>ca/en/adventures/gastronomic-marais-tour</t>
   </si>
   <si>
-    <t>2026-09-23T11:13:05.816Z</t>
+    <t>2026-09-23T14:53:09.542Z</t>
   </si>
   <si>
     <t>Gastronomic Marais Tour</t>
@@ -460,7 +463,7 @@
     <t>ca/en/adventures/napa-wine-tasting</t>
   </si>
   <si>
-    <t>2026-09-23T11:13:11.243Z</t>
+    <t>2026-09-23T14:53:14.064Z</t>
   </si>
   <si>
     <t>Napa Wine Tasting</t>
@@ -475,7 +478,7 @@
     <t>ca/en/adventures/riverside-camping-australia</t>
   </si>
   <si>
-    <t>2026-09-23T11:13:15.823Z</t>
+    <t>2026-09-23T14:53:18.736Z</t>
   </si>
   <si>
     <t>Riverside Camping</t>
@@ -490,7 +493,7 @@
     <t>ca/en/adventures/ski-touring-mont-blanc</t>
   </si>
   <si>
-    <t>2026-09-23T11:13:19.952Z</t>
+    <t>2026-09-23T14:53:22.836Z</t>
   </si>
   <si>
     <t>Ski Touring Mont Blanc</t>
@@ -505,7 +508,7 @@
     <t>ca/en/adventures/surf-camp-costa-rica</t>
   </si>
   <si>
-    <t>2026-09-23T11:13:27.781Z</t>
+    <t>2026-09-23T14:53:28.128Z</t>
   </si>
   <si>
     <t>Surf Camp in Costa Rica</t>
@@ -520,7 +523,7 @@
     <t>ca/en/adventures/tahoe-skiing</t>
   </si>
   <si>
-    <t>2026-09-23T11:13:33.091Z</t>
+    <t>2026-09-23T14:53:32.078Z</t>
   </si>
   <si>
     <t>Tahoe Skiing</t>
@@ -535,7 +538,7 @@
     <t>ca/en/adventures/west-coast-cycling</t>
   </si>
   <si>
-    <t>2026-09-23T11:13:39.038Z</t>
+    <t>2026-09-23T14:53:37.414Z</t>
   </si>
   <si>
     <t>West Coast Cycling</t>
@@ -550,7 +553,7 @@
     <t>ca/en/adventures/whistler-mountain-biking</t>
   </si>
   <si>
-    <t>2026-09-23T11:13:45.173Z</t>
+    <t>2026-09-23T14:53:41.886Z</t>
   </si>
   <si>
     <t>Whistler Mountain Biking</t>
@@ -565,7 +568,7 @@
     <t>ca/en/adventures/yosemite-backpacking</t>
   </si>
   <si>
-    <t>2026-09-23T11:13:51.047Z</t>
+    <t>2026-09-23T14:53:46.222Z</t>
   </si>
   <si>
     <t>Yosemite Backpacking</t>
@@ -679,7 +682,7 @@
     <t>us/en/adventures/bali-surf-camp</t>
   </si>
   <si>
-    <t>2026-09-23T11:11:06.753Z</t>
+    <t>2026-09-23T14:51:04.657Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/bali-surf-camp.html</t>
@@ -691,7 +694,7 @@
     <t>us/en/adventures/beervana-portland</t>
   </si>
   <si>
-    <t>2026-09-23T11:11:13.301Z</t>
+    <t>2026-09-23T14:51:09.273Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/beervana-portland.html</t>
@@ -703,7 +706,7 @@
     <t>us/en/adventures/climbing-new-zealand</t>
   </si>
   <si>
-    <t>2026-09-23T11:11:18.165Z</t>
+    <t>2026-09-23T14:51:14.374Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/climbing-new-zealand.html</t>
@@ -715,7 +718,7 @@
     <t>us/en/adventures/colorado-rock-climbing</t>
   </si>
   <si>
-    <t>2026-09-23T11:11:23.619Z</t>
+    <t>2026-09-23T14:51:18.935Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/colorado-rock-climbing.html</t>
@@ -727,7 +730,7 @@
     <t>us/en/adventures/cycling-southern-utah</t>
   </si>
   <si>
-    <t>2026-09-23T11:11:29.496Z</t>
+    <t>2026-09-23T14:51:25.203Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/cycling-southern-utah.html</t>
@@ -739,7 +742,7 @@
     <t>us/en/adventures/cycling-tuscany</t>
   </si>
   <si>
-    <t>2026-09-23T11:11:34.773Z</t>
+    <t>2026-09-23T14:51:30.172Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/cycling-tuscany.html</t>
@@ -751,7 +754,7 @@
     <t>us/en/adventures/downhill-skiing-wyoming</t>
   </si>
   <si>
-    <t>2026-09-23T11:11:40.072Z</t>
+    <t>2026-09-23T14:51:35.624Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/downhill-skiing-wyoming.html</t>
@@ -763,7 +766,7 @@
     <t>us/en/adventures/gastronomic-marais-tour</t>
   </si>
   <si>
-    <t>2026-09-23T11:11:44.368Z</t>
+    <t>2026-09-23T14:51:40.473Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/gastronomic-marais-tour.html</t>
@@ -775,7 +778,7 @@
     <t>us/en/adventures/napa-wine-tasting</t>
   </si>
   <si>
-    <t>2026-09-23T11:11:50.122Z</t>
+    <t>2026-09-23T14:51:46.587Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/napa-wine-tasting.html</t>
@@ -787,7 +790,7 @@
     <t>us/en/adventures/riverside-camping-australia</t>
   </si>
   <si>
-    <t>2026-09-23T11:11:55.587Z</t>
+    <t>2026-09-23T14:51:51.317Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/riverside-camping-australia.html</t>
@@ -799,7 +802,7 @@
     <t>us/en/adventures/ski-touring-mont-blanc</t>
   </si>
   <si>
-    <t>2026-09-23T11:12:00.736Z</t>
+    <t>2026-09-23T14:51:56.986Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/ski-touring-mont-blanc.html</t>
@@ -811,7 +814,7 @@
     <t>us/en/adventures/surf-camp-costa-rica</t>
   </si>
   <si>
-    <t>2026-09-23T11:12:05.562Z</t>
+    <t>2026-09-23T14:52:01.585Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/surf-camp-costa-rica.html</t>
@@ -823,7 +826,7 @@
     <t>us/en/adventures/tahoe-skiing</t>
   </si>
   <si>
-    <t>2026-09-23T11:12:10.002Z</t>
+    <t>2026-09-23T14:52:06.411Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/tahoe-skiing.html</t>
@@ -835,7 +838,7 @@
     <t>us/en/adventures/west-coast-cycling</t>
   </si>
   <si>
-    <t>2026-09-23T11:12:15.208Z</t>
+    <t>2026-09-23T14:52:11.100Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/west-coast-cycling.html</t>
@@ -847,7 +850,7 @@
     <t>us/en/adventures/whistler-mountain-biking</t>
   </si>
   <si>
-    <t>2026-09-23T11:12:19.705Z</t>
+    <t>2026-09-23T14:52:17.064Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/whistler-mountain-biking.html</t>
@@ -859,7 +862,7 @@
     <t>us/en/adventures/yosemite-backpacking</t>
   </si>
   <si>
-    <t>2026-09-23T11:12:24.490Z</t>
+    <t>2026-09-23T14:52:22.744Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/yosemite-backpacking.html</t>
@@ -1616,10 +1619,10 @@
         <v>53</v>
       </c>
       <c r="B11" t="s">
-        <v>9</v>
+        <v>54</v>
       </c>
       <c r="C11" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D11" t="s">
         <v>11</v>
@@ -1628,24 +1631,24 @@
         <v>12</v>
       </c>
       <c r="F11" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G11" t="s">
         <v>14</v>
       </c>
       <c r="H11" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B12" t="s">
         <v>17</v>
       </c>
       <c r="C12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D12" t="s">
         <v>11</v>
@@ -1654,1391 +1657,1391 @@
         <v>12</v>
       </c>
       <c r="F12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G12" t="s">
         <v>43</v>
       </c>
       <c r="H12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B13" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C13" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D13" t="s">
         <v>11</v>
       </c>
       <c r="E13" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F13" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G13" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B14" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D14" t="s">
         <v>11</v>
       </c>
       <c r="E14" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F14" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G14" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B15" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C15" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D15" t="s">
         <v>11</v>
       </c>
       <c r="E15" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F15" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G15" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H15" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B16" t="s">
         <v>17</v>
       </c>
       <c r="C16" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D16" t="s">
         <v>11</v>
       </c>
       <c r="E16" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F16" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G16" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H16" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B17" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C17" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D17" t="s">
         <v>11</v>
       </c>
       <c r="E17" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F17" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="G17" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H17" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B18" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C18" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D18" t="s">
         <v>11</v>
       </c>
       <c r="E18" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F18" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G18" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H18" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B19" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C19" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D19" t="s">
         <v>11</v>
       </c>
       <c r="E19" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F19" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G19" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H19" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B20" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C20" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D20" t="s">
         <v>11</v>
       </c>
       <c r="E20" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F20" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G20" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H20" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B21" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C21" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D21" t="s">
         <v>11</v>
       </c>
       <c r="E21" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F21" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G21" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H21" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B22" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C22" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D22" t="s">
         <v>11</v>
       </c>
       <c r="E22" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F22" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G22" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H22" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B23" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C23" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D23" t="s">
         <v>11</v>
       </c>
       <c r="E23" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F23" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G23" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H23" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B24" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C24" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D24" t="s">
         <v>11</v>
       </c>
       <c r="E24" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F24" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G24" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H24" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B25" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C25" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D25" t="s">
         <v>11</v>
       </c>
       <c r="E25" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F25" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G25" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H25" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B26" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C26" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D26" t="s">
         <v>11</v>
       </c>
       <c r="E26" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F26" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G26" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H26" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B27" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C27" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D27" t="s">
         <v>11</v>
       </c>
       <c r="E27" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F27" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G27" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H27" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B28" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C28" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D28" t="s">
         <v>11</v>
       </c>
       <c r="E28" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F28" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G28" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H28" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B29" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C29" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D29" t="s">
         <v>11</v>
       </c>
       <c r="E29" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F29" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G29" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H29" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B30" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C30" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D30" t="s">
         <v>11</v>
       </c>
       <c r="E30" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F30" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G30" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H30" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B31" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C31" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D31" t="s">
         <v>11</v>
       </c>
       <c r="E31" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F31" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G31" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H31" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B32" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C32" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D32" t="s">
         <v>11</v>
       </c>
       <c r="E32" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F32" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="G32" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="H32" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B33" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C33" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D33" t="s">
         <v>11</v>
       </c>
       <c r="E33" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F33" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="G33" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H33" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B34" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C34" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D34" t="s">
         <v>11</v>
       </c>
       <c r="E34" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F34" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="G34" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H34" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B35" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C35" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D35" t="s">
         <v>11</v>
       </c>
       <c r="E35" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F35" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="G35" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="H35" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B36" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C36" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D36" t="s">
         <v>11</v>
       </c>
       <c r="E36" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F36" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G36" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H36" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B37" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C37" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D37" t="s">
         <v>11</v>
       </c>
       <c r="E37" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F37" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G37" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="H37" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B38" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C38" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D38" t="s">
         <v>11</v>
       </c>
       <c r="E38" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F38" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="G38" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="H38" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B39" t="s">
         <v>17</v>
       </c>
       <c r="C39" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D39" t="s">
         <v>11</v>
       </c>
       <c r="E39" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F39" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="G39" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H39" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B40" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C40" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D40" t="s">
         <v>11</v>
       </c>
       <c r="E40" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F40" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="G40" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H40" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B41" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C41" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D41" t="s">
         <v>11</v>
       </c>
       <c r="E41" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F41" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G41" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="H41" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B42" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C42" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D42" t="s">
         <v>11</v>
       </c>
       <c r="E42" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F42" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="G42" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="H42" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B43" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C43" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D43" t="s">
         <v>11</v>
       </c>
       <c r="E43" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F43" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="G43" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H43" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B44" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C44" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D44" t="s">
         <v>11</v>
       </c>
       <c r="E44" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F44" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="G44" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H44" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B45" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C45" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D45" t="s">
         <v>11</v>
       </c>
       <c r="E45" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F45" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="G45" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H45" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B46" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C46" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D46" t="s">
         <v>11</v>
       </c>
       <c r="E46" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F46" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G46" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H46" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B47" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C47" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D47" t="s">
         <v>11</v>
       </c>
       <c r="E47" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F47" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="G47" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H47" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B48" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C48" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D48" t="s">
         <v>11</v>
       </c>
       <c r="E48" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F48" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="G48" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H48" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B49" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C49" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D49" t="s">
         <v>11</v>
       </c>
       <c r="E49" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F49" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G49" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H49" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B50" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C50" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D50" t="s">
         <v>11</v>
       </c>
       <c r="E50" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F50" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="G50" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H50" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B51" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C51" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D51" t="s">
         <v>11</v>
       </c>
       <c r="E51" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F51" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="G51" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H51" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B52" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C52" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D52" t="s">
         <v>11</v>
       </c>
       <c r="E52" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F52" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="G52" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H52" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B53" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C53" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D53" t="s">
         <v>11</v>
       </c>
       <c r="E53" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F53" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="G53" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H53" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B54" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C54" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D54" t="s">
         <v>11</v>
       </c>
       <c r="E54" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F54" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="G54" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="H54" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B55" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C55" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D55" t="s">
         <v>11</v>
       </c>
       <c r="E55" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F55" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="G55" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H55" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B56" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C56" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D56" t="s">
         <v>11</v>
       </c>
       <c r="E56" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F56" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="G56" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="H56" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B57" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C57" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D57" t="s">
         <v>11</v>
       </c>
       <c r="E57" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F57" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="G57" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="H57" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B58" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C58" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D58" t="s">
         <v>11</v>
       </c>
       <c r="E58" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F58" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="G58" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H58" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B59" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C59" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D59" t="s">
         <v>11</v>
       </c>
       <c r="E59" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F59" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="G59" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="H59" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B60" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C60" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D60" t="s">
         <v>11</v>
       </c>
       <c r="E60" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F60" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="G60" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="H60" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B61" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C61" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D61" t="s">
         <v>11</v>
       </c>
       <c r="E61" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F61" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="G61" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H61" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B62" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C62" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D62" t="s">
         <v>11</v>
       </c>
       <c r="E62" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F62" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="G62" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="H62" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B63" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C63" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D63" t="s">
         <v>11</v>
       </c>
       <c r="E63" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F63" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="G63" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="H63" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B64" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C64" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="D64" t="s">
         <v>11</v>
       </c>
       <c r="E64" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F64" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="G64" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="H64" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B65" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C65" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D65" t="s">
         <v>11</v>
       </c>
       <c r="E65" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F65" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="G65" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="H65" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
   </sheetData>

</xml_diff>